<commit_message>
Use real candidate names/parties in samples; make stat lookup label-based
- build_xlsx.py now finds Registered Voters/Rejected Ballots (and the
  other Summary key/value fields) by row label instead of a hardcoded
  cell reference, so it no longer breaks on inputs with a different
  Summary layout (e.g. sample-raw-export.xlsx no longer needs the
  original placeholder-row padding).
- Refreshed sample-raw-export.xlsx and both sample outputs to use real
  candidate names/parties instead of the earlier anonymized test data.
</commit_message>
<xml_diff>
--- a/tools/election-results-export/sample-output-formatted.xlsx
+++ b/tools/election-results-export/sample-output-formatted.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="47">
   <si>
     <t xml:space="preserve">BOZ ELECTION RESULTS</t>
   </si>
@@ -34,7 +34,7 @@
     <t xml:space="preserve">Presidential Election Results  |  National</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated: 7/6/2026, 8:39:20 PM</t>
+    <t xml:space="preserve">Generated: 7/7/2026, 9:00:00 AM</t>
   </si>
   <si>
     <t xml:space="preserve">PROJECTED WINNER</t>
@@ -82,49 +82,88 @@
     <t xml:space="preserve">Vote Share (%)</t>
   </si>
   <si>
-    <t xml:space="preserve">Candidate bm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">—</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Candidate hh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Candidate fm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Candidate hk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Candidate kbf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Candidate hkunda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Candidate xc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Candidate dp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Candidate rs2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Candidate aan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Candidate gk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Candidate gmc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Candidate rs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Candidate bmush</t>
+    <t xml:space="preserve">Mr Brian Mundubile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NRPUP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mr Hakainde Hichilema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UPND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr Fred M'membe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mr Harry Kalaba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mr Kelvin Fube Bwalya (KBF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZMP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mr Howard Kunda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZAWAPA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mr Xavier Chungu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LDP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr Dan Pule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CDP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mr Richwell Siamunene</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NFP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mr Ackim Antony Njobvu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ms Given Katuta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Independent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mr Given Mwenya Chansa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MEE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr Richard Silumbe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr Brian Mushimba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPP</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -145,7 +184,7 @@
   </numFmts>
   <fonts count="17">
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -757,14 +796,17 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
+                <a:shade val="94000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -851,8 +893,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
-  <sheetFormatPr defaultColWidth="8.62109375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="1" style="0" width="26"/>
   </cols>
@@ -896,12 +938,12 @@
     <row r="6" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="str">
         <f aca="false">INDEX(Results!B:B,MATCH(1,Results!A:A,0))</f>
-        <v>Candidate bm</v>
+        <v>Mr Brian Mundubile</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="7" t="n">
         <f aca="false">INDEX(Results!D:D,MATCH(1,Results!A:A,0))</f>
-        <v>1558</v>
+        <v>2178</v>
       </c>
       <c r="D6" s="7"/>
     </row>
@@ -910,7 +952,7 @@
       <c r="B7" s="6"/>
       <c r="C7" s="8" t="n">
         <f aca="false">INDEX(Results!E:E,MATCH(1,Results!A:A,0))</f>
-        <v>0.527420446851727</v>
+        <v>0.592814371257485</v>
       </c>
       <c r="D7" s="8"/>
     </row>
@@ -932,7 +974,7 @@
       </c>
       <c r="B10" s="10"/>
       <c r="C10" s="11" t="n">
-        <v>3460</v>
+        <v>4302</v>
       </c>
       <c r="D10" s="11"/>
     </row>
@@ -953,7 +995,7 @@
       <c r="B12" s="10"/>
       <c r="C12" s="14" t="n">
         <f aca="false">Results!$D$16</f>
-        <v>2954</v>
+        <v>3674</v>
       </c>
       <c r="D12" s="14"/>
     </row>
@@ -964,7 +1006,7 @@
       <c r="B13" s="12"/>
       <c r="C13" s="15" t="n">
         <f aca="false">C12+C11</f>
-        <v>2954</v>
+        <v>3674</v>
       </c>
       <c r="D13" s="15"/>
     </row>
@@ -975,7 +1017,7 @@
       <c r="B14" s="10"/>
       <c r="C14" s="16" t="n">
         <f aca="false">C13/C10</f>
-        <v>0.853757225433526</v>
+        <v>0.854021385402139</v>
       </c>
       <c r="D14" s="16"/>
     </row>
@@ -990,10 +1032,7 @@
       </c>
       <c r="D15" s="17"/>
     </row>
-    <row r="16" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4"/>
-    </row>
+    <row r="16" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
         <v>11</v>
@@ -1002,7 +1041,7 @@
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
     </row>
-    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
         <v>12</v>
       </c>
@@ -1016,47 +1055,47 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="n">
         <v>1</v>
       </c>
       <c r="B19" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Results!B:B,MATCH(1,Results!A:A,0)),"")</f>
-        <v>Candidate bm</v>
+        <v>Mr Brian Mundubile</v>
       </c>
       <c r="C19" s="21" t="n">
         <f aca="false">IFERROR(INDEX(Results!D:D,MATCH(1,Results!A:A,0)),"")</f>
-        <v>1558</v>
+        <v>2178</v>
       </c>
       <c r="D19" s="22" t="n">
         <f aca="false">IFERROR(INDEX(Results!E:E,MATCH(1,Results!A:A,0)),"")</f>
-        <v>0.527420446851727</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>0.592814371257485</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="23" t="n">
         <v>2</v>
       </c>
       <c r="B20" s="24" t="str">
         <f aca="false">IFERROR(INDEX(Results!B:B,MATCH(2,Results!A:A,0)),"")</f>
-        <v>Candidate hh</v>
+        <v>Mr Hakainde Hichilema</v>
       </c>
       <c r="C20" s="25" t="n">
         <f aca="false">IFERROR(INDEX(Results!D:D,MATCH(2,Results!A:A,0)),"")</f>
-        <v>1101</v>
+        <v>1201</v>
       </c>
       <c r="D20" s="26" t="n">
         <f aca="false">IFERROR(INDEX(Results!E:E,MATCH(2,Results!A:A,0)),"")</f>
-        <v>0.372714962762356</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>0.326891671203048</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="n">
         <v>3</v>
       </c>
       <c r="B21" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Results!B:B,MATCH(3,Results!A:A,0)),"")</f>
-        <v>Candidate fm</v>
+        <v>Dr Fred M'membe</v>
       </c>
       <c r="C21" s="21" t="n">
         <f aca="false">IFERROR(INDEX(Results!D:D,MATCH(3,Results!A:A,0)),"")</f>
@@ -1064,20 +1103,8 @@
       </c>
       <c r="D21" s="22" t="n">
         <f aca="false">IFERROR(INDEX(Results!E:E,MATCH(3,Results!A:A,0)),"")</f>
-        <v>0.0233581584292485</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-    </row>
-    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4"/>
-      <c r="B23" s="4"/>
-    </row>
-    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4"/>
-      <c r="B24" s="4"/>
+        <v>0.0187806205770278</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="21">
@@ -1119,7 +1146,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultColWidth="8.62109375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
@@ -1144,7 +1171,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="n">
         <v>1</v>
       </c>
@@ -1155,14 +1182,14 @@
         <v>19</v>
       </c>
       <c r="D2" s="30" t="n">
-        <v>1558</v>
+        <v>2178</v>
       </c>
       <c r="E2" s="31" t="n">
         <f aca="false">D2/D$16</f>
-        <v>0.527420446851727</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>0.592814371257485</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="32" t="n">
         <v>2</v>
       </c>
@@ -1170,241 +1197,241 @@
         <v>20</v>
       </c>
       <c r="C3" s="33" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D3" s="34" t="n">
-        <v>1101</v>
+        <v>1201</v>
       </c>
       <c r="E3" s="35" t="n">
         <f aca="false">D3/D$16</f>
-        <v>0.372714962762356</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>0.326891671203048</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="36" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="37" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" s="37" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D4" s="38" t="n">
         <v>69</v>
       </c>
       <c r="E4" s="39" t="n">
         <f aca="false">D4/D$16</f>
-        <v>0.0233581584292485</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>0.0187806205770278</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="D5" s="34" t="n">
         <v>55</v>
       </c>
       <c r="E5" s="35" t="n">
         <f aca="false">D5/D$16</f>
-        <v>0.0186188219363575</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>0.0149700598802395</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="36" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="D6" s="38" t="n">
         <v>25</v>
       </c>
       <c r="E6" s="39" t="n">
         <f aca="false">D6/D$16</f>
-        <v>0.00846310088016249</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>0.00680457267283615</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="D7" s="34" t="n">
         <v>20</v>
       </c>
       <c r="E7" s="35" t="n">
         <f aca="false">D7/D$16</f>
-        <v>0.00677048070412999</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>0.00544365813826892</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="36" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C8" s="37" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="D8" s="38" t="n">
         <v>20</v>
       </c>
       <c r="E8" s="39" t="n">
         <f aca="false">D8/D$16</f>
-        <v>0.00677048070412999</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>0.00544365813826892</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="D9" s="34" t="n">
         <v>20</v>
       </c>
       <c r="E9" s="35" t="n">
         <f aca="false">D9/D$16</f>
-        <v>0.00677048070412999</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>0.00544365813826892</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="36" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="D10" s="38" t="n">
         <v>20</v>
       </c>
       <c r="E10" s="39" t="n">
         <f aca="false">D10/D$16</f>
-        <v>0.00677048070412999</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>0.00544365813826892</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="D11" s="34" t="n">
         <v>19</v>
       </c>
       <c r="E11" s="35" t="n">
         <f aca="false">D11/D$16</f>
-        <v>0.00643195666892349</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>0.00517147523135547</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="36" t="n">
         <v>11</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="C12" s="37" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D12" s="38" t="n">
         <v>14</v>
       </c>
       <c r="E12" s="39" t="n">
         <f aca="false">D12/D$16</f>
-        <v>0.004739336492891</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>0.00381056069678824</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="D13" s="34" t="n">
         <v>11</v>
       </c>
       <c r="E13" s="35" t="n">
         <f aca="false">D13/D$16</f>
-        <v>0.0037237643872715</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>0.0029940119760479</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="36" t="n">
         <v>13</v>
       </c>
       <c r="B14" s="37" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="C14" s="37" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="D14" s="38" t="n">
         <v>11</v>
       </c>
       <c r="E14" s="39" t="n">
         <f aca="false">D14/D$16</f>
-        <v>0.0037237643872715</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>0.0029940119760479</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="D15" s="34" t="n">
         <v>11</v>
       </c>
       <c r="E15" s="35" t="n">
         <f aca="false">D15/D$16</f>
-        <v>0.0037237643872715</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>0.0029940119760479</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="40"/>
       <c r="B16" s="40"/>
       <c r="C16" s="41" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D16" s="42" t="n">
         <f aca="false">SUM(D2:D15)</f>
-        <v>2954</v>
+        <v>3674</v>
       </c>
       <c r="E16" s="43" t="n">
         <f aca="false">D16/D16</f>
@@ -1422,7 +1449,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{704C1456-86F7-4511-90E1-5FA563222645}</x14:id>
+          <x14:id>{805B3A94-2460-426A-BC19-238726ED45A2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -1439,7 +1466,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{704C1456-86F7-4511-90E1-5FA563222645}">
+          <x14:cfRule type="dataBar" id="{805B3A94-2460-426A-BC19-238726ED45A2}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>